<commit_message>
Night 21.09: pupil 1v1 vs stand, synced teacher grid (193 fixes), rebuilt load, greedy 837/893 + draft export
</commit_message>
<xml_diff>
--- a/данные/тест_реал/РеальнаяНагрузка_5-11.xlsx
+++ b/данные/тест_реал/РеальнаяНагрузка_5-11.xlsx
@@ -726,7 +726,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Коротченя С.И.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Коротченя С.И.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
@@ -1143,7 +1143,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Королёнок У.С.</t>
+          <t>Авдеёнок О.В.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr"/>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Королёнок У.С.</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
@@ -1514,7 +1514,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Авдеёнок О.В.</t>
+          <t>Королёнок У.С.</t>
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Александрович В.А.</t>
+          <t>Пекарский И.В.</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -2089,7 +2089,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Лабикова Н.К.</t>
+          <t>Лащ А.Н.</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Гордионок С.Г.</t>
+          <t>Хинич К.Н.</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Новикова И.А.</t>
+          <t>Павлович С.А.</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -2630,7 +2630,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Лабикова Н.К.</t>
+          <t>Лащ А.Н.</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -2893,7 +2893,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Потапов В.Н.</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -3082,7 +3082,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Лащ А.Н.</t>
+          <t>Павлович С.А.</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
@@ -3109,7 +3109,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Лабикова Н.К.</t>
+          <t>Лащ А.Н.</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -3179,7 +3179,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Бадеева Е.В.</t>
+          <t>Авхименко Е.С.</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
@@ -3395,7 +3395,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Лабикова Н.К.</t>
+          <t>Лащ А.Н.</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -3405,7 +3405,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Гордионок С.Г.</t>
+          <t>Хинич К.Н.</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -3604,7 +3604,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Павлович С.А.</t>
         </is>
       </c>
       <c r="E113" t="inlineStr"/>
@@ -3975,7 +3975,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Дамашевич Е.С.</t>
         </is>
       </c>
       <c r="E126" t="inlineStr"/>
@@ -4056,7 +4056,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Александрович В.А.</t>
+          <t>Шаройкина А.В.</t>
         </is>
       </c>
       <c r="E129" t="inlineStr"/>
@@ -4199,7 +4199,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Шаройкина А.В.</t>
         </is>
       </c>
       <c r="E134" t="inlineStr"/>
@@ -5014,7 +5014,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Александрович В.А.</t>
+          <t>Шаройкина А.В.</t>
         </is>
       </c>
       <c r="E163" t="inlineStr"/>
@@ -5250,7 +5250,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Замена (вакансия)</t>
+          <t>Шаройкина А.В.</t>
         </is>
       </c>
       <c r="E171" t="inlineStr"/>
@@ -5404,7 +5404,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Хильчук В.В.</t>
+          <t>Сидорович С.Б.</t>
         </is>
       </c>
       <c r="E177" t="inlineStr"/>
@@ -5458,7 +5458,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Сидорович С.Б.</t>
+          <t>Крупович Ю.А.</t>
         </is>
       </c>
       <c r="E179" t="inlineStr"/>
@@ -5512,7 +5512,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Свищёва В.А.</t>
         </is>
       </c>
       <c r="E181" t="inlineStr"/>
@@ -7706,17 +7706,17 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
+          <t>Лащ А.Н.</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>A/B</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
           <t>Лабикова Н.К.</t>
-        </is>
-      </c>
-      <c r="E259" t="inlineStr">
-        <is>
-          <t>A/B</t>
-        </is>
-      </c>
-      <c r="F259" t="inlineStr">
-        <is>
-          <t>ВАКАНСИЯ (пара)</t>
         </is>
       </c>
       <c r="G259" t="inlineStr">
@@ -7876,7 +7876,7 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>Павлович С.А.</t>
+          <t>Крупович Ю.А.</t>
         </is>
       </c>
       <c r="E265" t="inlineStr"/>
@@ -8347,17 +8347,17 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
+          <t>Лащ А.Н.</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>A/B</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
           <t>Лабикова Н.К.</t>
-        </is>
-      </c>
-      <c r="E282" t="inlineStr">
-        <is>
-          <t>A/B</t>
-        </is>
-      </c>
-      <c r="F282" t="inlineStr">
-        <is>
-          <t>ВАКАНСИЯ (пара)</t>
         </is>
       </c>
       <c r="G282" t="inlineStr">
@@ -8772,17 +8772,17 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
+          <t>Лащ А.Н.</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>A/B</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
           <t>Лабикова Н.К.</t>
-        </is>
-      </c>
-      <c r="E297" t="inlineStr">
-        <is>
-          <t>A/B</t>
-        </is>
-      </c>
-      <c r="F297" t="inlineStr">
-        <is>
-          <t>ВАКАНСИЯ (пара)</t>
         </is>
       </c>
       <c r="G297" t="inlineStr">
@@ -9332,17 +9332,17 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
+          <t>Лащ А.Н.</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>A/B</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
           <t>Лабикова Н.К.</t>
-        </is>
-      </c>
-      <c r="E317" t="inlineStr">
-        <is>
-          <t>A/B</t>
-        </is>
-      </c>
-      <c r="F317" t="inlineStr">
-        <is>
-          <t>ВАКАНСИЯ (пара)</t>
         </is>
       </c>
       <c r="G317" t="inlineStr">
@@ -9695,7 +9695,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Денискин Е.В.</t>
+          <t>Замена (вакансия)</t>
         </is>
       </c>
       <c r="E330" t="inlineStr"/>
@@ -10329,7 +10329,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>Денискин Е.В.</t>
+          <t>Замена (вакансия)</t>
         </is>
       </c>
       <c r="E352" t="inlineStr"/>
@@ -10761,7 +10761,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>Денискин Е.В.</t>
+          <t>Замена (вакансия)</t>
         </is>
       </c>
       <c r="E368" t="inlineStr"/>
@@ -11453,7 +11453,7 @@
       </c>
       <c r="D392" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Замена (вакансия)</t>
         </is>
       </c>
       <c r="E392" t="inlineStr"/>
@@ -11480,7 +11480,7 @@
       </c>
       <c r="D393" t="inlineStr">
         <is>
-          <t>Денискин Е.В.</t>
+          <t>Замена (вакансия)</t>
         </is>
       </c>
       <c r="E393" t="inlineStr"/>

</xml_diff>

<commit_message>
22-23.09: demo v 1 klik, krasivyy dashboard, teacher-gap optimizatsiya 377->265, realnyy load (Denis 14ch, Gorodionok/Pluzhnikova); suit 317+2/0
</commit_message>
<xml_diff>
--- a/данные/тест_реал/РеальнаяНагрузка_5-11.xlsx
+++ b/данные/тест_реал/РеальнаяНагрузка_5-11.xlsx
@@ -583,7 +583,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Шустова В.Д.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -593,7 +593,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Богданова К.Ю.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -896,7 +896,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Шустова В.Д.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Богданова К.Ю.</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1425,7 +1425,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Шустова В.Д.</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1435,7 +1435,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Богданова К.Ю.</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Шустова В.Д.</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -1825,7 +1825,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Богданова К.Ю.</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2178,7 +2178,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Новикова И.А.</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2188,7 +2188,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Островская В.В.</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -2267,7 +2267,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Бадеева Е.В.</t>
+          <t>Чепикова У.В.</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Бадеева Е.В.</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Наконечная Е.В.</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Новикова И.А.</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -2393,7 +2393,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Островская В.В.</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Бадеева Е.В.</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Наконечная Е.В.</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -2781,7 +2781,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Плужникова М.Д.</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -2791,7 +2791,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Хорошко Е.Н.</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -3055,7 +3055,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Плужнова М.Д.</t>
+          <t>Плужникова М.Д.</t>
         </is>
       </c>
       <c r="E94" t="inlineStr"/>
@@ -3144,7 +3144,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Бадеева Е.В.</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -3154,7 +3154,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Наконечная Е.В.</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -3453,7 +3453,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Плужникова М.Д.</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -3463,7 +3463,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Хорошко Е.Н.</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -3569,7 +3569,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Бадеева Е.В.</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -3579,7 +3579,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Наконечная Е.В.</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -3739,7 +3739,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Разводовская М.О.</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -3749,7 +3749,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Богданова К.Ю.</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -3797,7 +3797,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Бадеева Е.В.</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Наконечная Е.В.</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -3948,7 +3948,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Замена (вакансия)</t>
+          <t>Городионок С.Г.</t>
         </is>
       </c>
       <c r="E125" t="inlineStr"/>
@@ -4137,7 +4137,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Бадеева Е.В.</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -4147,7 +4147,7 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Наконечная Е.В.</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
@@ -4280,7 +4280,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Разводовская М.О.</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Островская В.В.</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
@@ -4342,7 +4342,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Наконечная Е.В.</t>
+          <t>Городионок С.Г.</t>
         </is>
       </c>
       <c r="E139" t="inlineStr"/>
@@ -4705,7 +4705,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Плужникова М.Д.</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -4715,7 +4715,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Островская В.В.</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -4767,7 +4767,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Бадеева Е.В.</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
@@ -4777,7 +4777,7 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Наконечная Е.В.</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
@@ -5612,7 +5612,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Шустова В.Д.</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
@@ -5622,7 +5622,7 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Новикова И.А.</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
@@ -5647,7 +5647,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Бадеева Е.В.</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
@@ -5657,7 +5657,7 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Наконечная Е.В.</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Гордионок С.Г.</t>
+          <t>Городионок С.Г.</t>
         </is>
       </c>
       <c r="E199" t="inlineStr"/>
@@ -6172,7 +6172,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Касперович А.А.</t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
@@ -6182,7 +6182,7 @@
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Островская В.В.</t>
         </is>
       </c>
       <c r="G205" t="inlineStr">
@@ -6261,7 +6261,7 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Бадеева Е.В.</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
@@ -6271,7 +6271,7 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Наконечная Е.В.</t>
         </is>
       </c>
       <c r="G208" t="inlineStr">
@@ -6609,7 +6609,7 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Касперович А.А.</t>
         </is>
       </c>
       <c r="E220" t="inlineStr">
@@ -6619,7 +6619,7 @@
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Островская В.В.</t>
         </is>
       </c>
       <c r="G220" t="inlineStr">
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Бадеева Е.В.</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Наконечная Е.В.</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
@@ -7192,7 +7192,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Шустова В.Д.</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
@@ -7202,7 +7202,7 @@
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Новикова И.А.</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
@@ -7335,7 +7335,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Бадеева Е.В.</t>
         </is>
       </c>
       <c r="E246" t="inlineStr">
@@ -7345,7 +7345,7 @@
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Наконечная Е.В.</t>
         </is>
       </c>
       <c r="G246" t="inlineStr">
@@ -7501,7 +7501,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Бадеева Е.В.</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
@@ -7511,7 +7511,7 @@
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Наконечная Е.В.</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
@@ -7536,7 +7536,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Касперович А.А.</t>
         </is>
       </c>
       <c r="E253" t="inlineStr">
@@ -7546,7 +7546,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Богданова К.Ю.</t>
         </is>
       </c>
       <c r="G253" t="inlineStr">
@@ -7957,7 +7957,7 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Бадеева Е.В.</t>
         </is>
       </c>
       <c r="E268" t="inlineStr">
@@ -7967,7 +7967,7 @@
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Наконечная Е.В.</t>
         </is>
       </c>
       <c r="G268" t="inlineStr">
@@ -8312,7 +8312,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Касперович А.А.</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -8322,7 +8322,7 @@
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Новикова И.А.</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">
@@ -8513,7 +8513,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Бадеева Е.В.</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -8523,7 +8523,7 @@
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Наконечная Е.В.</t>
         </is>
       </c>
       <c r="G288" t="inlineStr">
@@ -8602,7 +8602,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Новикова И.А.</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -8612,7 +8612,7 @@
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Хорошко Е.Н.</t>
         </is>
       </c>
       <c r="G291" t="inlineStr">
@@ -9050,7 +9050,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Бадеева Е.В.</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -9060,7 +9060,7 @@
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Наконечная Е.В.</t>
         </is>
       </c>
       <c r="G307" t="inlineStr">
@@ -9216,7 +9216,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Разводовская М.О.</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -9226,7 +9226,7 @@
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Касперович А.А.</t>
         </is>
       </c>
       <c r="G313" t="inlineStr">
@@ -9695,7 +9695,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Замена (вакансия)</t>
+          <t>Денискин Е.В.</t>
         </is>
       </c>
       <c r="E330" t="inlineStr"/>
@@ -9749,7 +9749,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Воробьёва Ж.А.</t>
+          <t>Липницкая М.И.</t>
         </is>
       </c>
       <c r="E332" t="inlineStr"/>
@@ -9911,7 +9911,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Хорошко Е.Н.</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
@@ -9921,7 +9921,7 @@
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Островская В.В.</t>
         </is>
       </c>
       <c r="G338" t="inlineStr">
@@ -10027,7 +10027,7 @@
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Бадеева Е.В.</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
@@ -10037,7 +10037,7 @@
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Наконечная Е.В.</t>
         </is>
       </c>
       <c r="G342" t="inlineStr">
@@ -10154,16 +10154,8 @@
           <t>Хорошко Е.Н.</t>
         </is>
       </c>
-      <c r="E346" t="inlineStr">
-        <is>
-          <t>A/B</t>
-        </is>
-      </c>
-      <c r="F346" t="inlineStr">
-        <is>
-          <t>ВАКАНСИЯ (пара)</t>
-        </is>
-      </c>
+      <c r="E346" t="inlineStr"/>
+      <c r="F346" t="inlineStr"/>
       <c r="G346" t="inlineStr">
         <is>
           <t>207</t>
@@ -10186,7 +10178,7 @@
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Бадеева Е.В.</t>
         </is>
       </c>
       <c r="E347" t="inlineStr">
@@ -10196,7 +10188,7 @@
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Наконечная Е.В.</t>
         </is>
       </c>
       <c r="G347" t="inlineStr">
@@ -10329,7 +10321,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>Замена (вакансия)</t>
+          <t>Денискин Е.В.</t>
         </is>
       </c>
       <c r="E352" t="inlineStr"/>
@@ -10537,11 +10529,11 @@
         </is>
       </c>
       <c r="C360" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>Гордионок С.Г.</t>
+          <t>Городионок С.Г.</t>
         </is>
       </c>
       <c r="E360" t="inlineStr"/>
@@ -10761,7 +10753,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>Замена (вакансия)</t>
+          <t>Денискин Е.В.</t>
         </is>
       </c>
       <c r="E368" t="inlineStr"/>
@@ -10788,7 +10780,7 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Денискин Е.В.</t>
         </is>
       </c>
       <c r="E369" t="inlineStr"/>
@@ -11047,7 +11039,7 @@
       </c>
       <c r="D378" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Бадеева Е.В.</t>
         </is>
       </c>
       <c r="E378" t="inlineStr">
@@ -11057,7 +11049,7 @@
       </c>
       <c r="F378" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Наконечная Е.В.</t>
         </is>
       </c>
       <c r="G378" t="inlineStr">
@@ -11082,7 +11074,7 @@
       </c>
       <c r="D379" t="inlineStr">
         <is>
-          <t>Воробьёва Ж.А.</t>
+          <t>Липницкая М.И.</t>
         </is>
       </c>
       <c r="E379" t="inlineStr"/>
@@ -11302,7 +11294,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Бадеева Е.В.</t>
         </is>
       </c>
       <c r="E387" t="inlineStr">
@@ -11312,7 +11304,7 @@
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Наконечная Е.В.</t>
         </is>
       </c>
       <c r="G387" t="inlineStr">
@@ -11418,7 +11410,7 @@
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ</t>
+          <t>Хорошко Е.Н.</t>
         </is>
       </c>
       <c r="E391" t="inlineStr">
@@ -11428,7 +11420,7 @@
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t>ВАКАНСИЯ (пара)</t>
+          <t>Островская В.В.</t>
         </is>
       </c>
       <c r="G391" t="inlineStr">
@@ -11453,7 +11445,7 @@
       </c>
       <c r="D392" t="inlineStr">
         <is>
-          <t>Замена (вакансия)</t>
+          <t>Денискин Е.В.</t>
         </is>
       </c>
       <c r="E392" t="inlineStr"/>
@@ -11480,7 +11472,7 @@
       </c>
       <c r="D393" t="inlineStr">
         <is>
-          <t>Замена (вакансия)</t>
+          <t>Денискин Е.В.</t>
         </is>
       </c>
       <c r="E393" t="inlineStr"/>

</xml_diff>